<commit_message>
修改t_analysis_date → t_start_date + t_end_date
</commit_message>
<xml_diff>
--- a/我的自选.xlsx
+++ b/我的自选.xlsx
@@ -29,12 +29,33 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
-    <t>序号</t>
+    <t>stocks</t>
   </si>
   <si>
-    <t>股票</t>
+    <t>start_date</t>
+  </si>
+  <si>
+    <t>end_date</t>
+  </si>
+  <si>
+    <t>t_start_date</t>
+  </si>
+  <si>
+    <t>t_end_date</t>
+  </si>
+  <si>
+    <t>神火股份</t>
+  </si>
+  <si>
+    <t>云铝股份</t>
+  </si>
+  <si>
+    <t>云天化</t>
+  </si>
+  <si>
+    <t>珀莱雅</t>
   </si>
 </sst>
 </file>
@@ -57,7 +78,7 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -402,27 +423,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -549,7 +555,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
@@ -561,34 +567,34 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="0">
@@ -673,17 +679,23 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -997,105 +1009,114 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="1"/>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="10.2300884955752" style="1" customWidth="1"/>
-    <col min="2" max="2" width="16.2035398230088" style="1" customWidth="1"/>
+    <col min="1" max="1" width="26.9557522123894" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7345132743363" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.3362831858407" style="2" customWidth="1"/>
+    <col min="4" max="4" width="27.2212389380531" style="2" customWidth="1"/>
+    <col min="5" max="5" width="18.858407079646" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:2">
-      <c r="A1" s="2" t="s">
+    <row r="1" ht="17.6" spans="1:5">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" ht="18" customHeight="1" spans="1:2">
-      <c r="A2" s="3">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3"/>
+    <row r="2" ht="22" customHeight="1" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="5">
+        <v>43831</v>
+      </c>
+      <c r="C2" s="5">
+        <v>46164</v>
+      </c>
+      <c r="D2" s="5">
+        <v>45292</v>
+      </c>
+      <c r="E2" s="5">
+        <v>46163</v>
+      </c>
     </row>
-    <row r="3" ht="18" customHeight="1" spans="1:2">
-      <c r="A3" s="3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3"/>
+    <row r="3" ht="22" customHeight="1" spans="1:5">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="5">
+        <v>43831</v>
+      </c>
+      <c r="C3" s="5">
+        <v>46164</v>
+      </c>
+      <c r="D3" s="5">
+        <v>45292</v>
+      </c>
+      <c r="E3" s="5">
+        <v>46163</v>
+      </c>
     </row>
-    <row r="4" ht="18" customHeight="1" spans="1:2">
-      <c r="A4" s="3">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3"/>
+    <row r="4" ht="22" customHeight="1" spans="1:5">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="5">
+        <v>43831</v>
+      </c>
+      <c r="C4" s="5">
+        <v>46164</v>
+      </c>
+      <c r="D4" s="5">
+        <v>45292</v>
+      </c>
+      <c r="E4" s="5">
+        <v>46163</v>
+      </c>
     </row>
-    <row r="5" ht="18" customHeight="1" spans="1:2">
-      <c r="A5" s="3">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3"/>
+    <row r="5" ht="22" customHeight="1" spans="1:5">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="5">
+        <v>43831</v>
+      </c>
+      <c r="C5" s="5">
+        <v>46164</v>
+      </c>
+      <c r="D5" s="5">
+        <v>45292</v>
+      </c>
+      <c r="E5" s="5">
+        <v>46163</v>
+      </c>
     </row>
-    <row r="6" ht="18" customHeight="1" spans="1:2">
-      <c r="A6" s="3">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3"/>
-    </row>
-    <row r="7" ht="18" customHeight="1" spans="1:2">
-      <c r="A7" s="3">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3"/>
-    </row>
-    <row r="8" ht="18" customHeight="1" spans="1:2">
-      <c r="A8" s="3">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3"/>
-    </row>
-    <row r="9" ht="18" customHeight="1" spans="1:2">
-      <c r="A9" s="3">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3"/>
-    </row>
-    <row r="10" ht="18" customHeight="1" spans="1:2">
-      <c r="A10" s="3">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3"/>
-    </row>
-    <row r="11" ht="18" customHeight="1" spans="1:2">
-      <c r="A11" s="3">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3"/>
-    </row>
-    <row r="12" ht="18" customHeight="1" spans="1:2">
-      <c r="A12" s="3">
-        <v>11</v>
-      </c>
-      <c r="B12" s="3"/>
-    </row>
-    <row r="13" ht="18" customHeight="1" spans="1:2">
-      <c r="A13" s="3">
-        <v>12</v>
-      </c>
-      <c r="B13" s="3"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" spans="1:2">
-      <c r="A14" s="3">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3"/>
-    </row>
-    <row r="15" ht="18" customHeight="1" spans="1:2">
-      <c r="A15" s="3">
-        <v>14</v>
-      </c>
-      <c r="B15" s="3"/>
-    </row>
+    <row r="6" ht="18" customHeight="1"/>
+    <row r="7" ht="18" customHeight="1"/>
+    <row r="8" ht="18" customHeight="1"/>
+    <row r="9" ht="18" customHeight="1"/>
+    <row r="10" ht="18" customHeight="1"/>
+    <row r="11" ht="18" customHeight="1"/>
+    <row r="12" ht="18" customHeight="1"/>
+    <row r="13" ht="18" customHeight="1"/>
+    <row r="14" ht="18" customHeight="1"/>
+    <row r="15" ht="18" customHeight="1"/>
+    <row r="16" ht="18" customHeight="1"/>
+    <row r="17" ht="18" customHeight="1"/>
+    <row r="18" ht="18" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>